<commit_message>
Main board manufacturing file generated and added
</commit_message>
<xml_diff>
--- a/SensWear-V1R1-Main/Output/Manufacturing/Assembly/Bill of Materials/Bill of Materials-SensWear-V1R1-MainBoard.xlsx
+++ b/SensWear-V1R1-Main/Output/Manufacturing/Assembly/Bill of Materials/Bill of Materials-SensWear-V1R1-MainBoard.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WORK\Projects\OpenRing\Hardware\OpenRing-V1R1-Main\Output\Manufacturing\Assembly\Bill of Materials\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WORK\Projects\OpenRing\Hardware\SensWear-V1R1-Main\Output\Manufacturing\Assembly\Bill of Materials\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{52B912FC-5738-45B0-BACA-D6839B10CAE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7AB2388D-7BF8-4EDF-BCC4-F089DBD8151A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4290" yWindow="4290" windowWidth="28800" windowHeight="15285" xr2:uid="{162A4FFF-0067-4B5F-86AD-896E5CB27ED7}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{07270503-5351-47F7-9BC7-9D25E3D2FE9D}"/>
   </bookViews>
   <sheets>
-    <sheet name="Bill of Materials-OpenRing-V1R1" sheetId="1" r:id="rId1"/>
+    <sheet name="Bill of Materials-SensWear-V1R1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Bill of Materials-OpenRing-V1R1'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Bill of Materials-SensWear-V1R1'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -1034,7 +1034,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74A6FFFF-BAAE-403D-9799-9A8DF614A7A9}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{634643FE-CF66-493D-ACC4-FAFAB62CB7CA}">
   <dimension ref="A1:I39"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>

</xml_diff>